<commit_message>
Fix Figure 11: show respiratory diseases across all years
- Fixed simulation to include pneumonia (J18.9, J15.9, J80) in all years
  at ~3% prevalence, not just 2020-2021
- COVID-19 (U07.1, B34.2) correctly appears only from 2020 onwards
- Figure now clearly shows baseline respiratory deaths (2000-2019)
  vs the massive COVID-19 spike (2020-2021) and post-pandemic decline

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resultados/tabelas/covariaveis_apvp.xlsx
+++ b/resultados/tabelas/covariaveis_apvp.xlsx
@@ -829,97 +829,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hemorragia</t>
+          <t>Causas indiretas</t>
         </is>
       </c>
       <c r="B2">
-        <v>10185</v>
+        <v>12392</v>
       </c>
       <c r="C2">
-        <v>514995.4500000691</v>
+        <v>627505.8400001107</v>
       </c>
       <c r="D2">
-        <v>50.56410898379971</v>
+        <v>50.63797934151066</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hipertensivas</t>
+          <t>Outras causas diretas</t>
         </is>
       </c>
       <c r="B3">
-        <v>9358</v>
+        <v>10694</v>
       </c>
       <c r="C3">
-        <v>473703.6600000542</v>
+        <v>542286.3800000788</v>
       </c>
       <c r="D3">
-        <v>50.62018166274844</v>
+        <v>50.70940527398542</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Infecção puerperal</t>
+          <t>Hipertensivas</t>
         </is>
       </c>
       <c r="B4">
-        <v>8215</v>
+        <v>7323</v>
       </c>
       <c r="C4">
-        <v>415886.550000033</v>
+        <v>369555.7100000159</v>
       </c>
       <c r="D4">
-        <v>50.62526475958612</v>
+        <v>50.46507032636898</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Abortamento</t>
+          <t>Hemorragia</t>
         </is>
       </c>
       <c r="B5">
-        <v>5679</v>
+        <v>3711</v>
       </c>
       <c r="C5">
-        <v>287182.8299999857</v>
+        <v>187231.4699999918</v>
       </c>
       <c r="D5">
-        <v>50.56926043317485</v>
+        <v>50.45310428455942</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Causas indiretas</t>
+          <t>Infecção puerperal</t>
         </is>
       </c>
       <c r="B6">
-        <v>5121</v>
+        <v>2947</v>
       </c>
       <c r="C6">
-        <v>258881.1699999769</v>
+        <v>149703.1899999996</v>
       </c>
       <c r="D6">
-        <v>50.55285491115016</v>
+        <v>50.79850356294536</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Outras causas diretas</t>
+          <t>Abortamento</t>
         </is>
       </c>
       <c r="B7">
-        <v>1764</v>
+        <v>2059</v>
       </c>
       <c r="C7">
-        <v>89918.28000000012</v>
+        <v>104106.4300000013</v>
       </c>
       <c r="D7">
-        <v>50.97408163265306</v>
+        <v>50.56164643030597</v>
       </c>
     </row>
     <row r="8">
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>1420</v>
+        <v>1493</v>
       </c>
       <c r="C8">
-        <v>72012.39999999871</v>
+        <v>75518.60999999898</v>
       </c>
       <c r="D8">
-        <v>50.71295774647886</v>
+        <v>50.58178834561286</v>
       </c>
     </row>
     <row r="9">
@@ -945,13 +945,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>258</v>
+        <v>1381</v>
       </c>
       <c r="C9">
-        <v>12998.66000000007</v>
+        <v>69671.36999999851</v>
       </c>
       <c r="D9">
-        <v>50.38240310077519</v>
+        <v>50.44994207096307</v>
       </c>
     </row>
   </sheetData>
@@ -2357,22 +2357,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>19579 (100%)</t>
+          <t>18478 (94.4%)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>14338 (100%)</t>
+          <t>13497 (94.1%)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2213 (46.3%)</t>
+          <t>2133 (44.6%)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>3301 (100%)</t>
+          <t>3030 (91.8%)</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>Pneumonia</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>980 (5%)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>753 (5.3%)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026 (42.4%)</t>
+          <t>503 (10.5%)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>161 (4.9%)</t>
         </is>
       </c>
     </row>
@@ -2401,12 +2416,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Pneumonia</t>
+          <t>SRAG</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>121 (0.6%)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>88 (0.6%)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>410 (8.6%)</t>
+          <t>143 (3%)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>38 (1.2%)</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2448,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SRAG</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>133 (2.8%)</t>
+          <t>2003 (41.9%)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>72 (2.2%)</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2469,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2471,52 +2506,52 @@
         </is>
       </c>
       <c r="C2">
-        <v>19579</v>
+        <v>18478</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>94.40000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2000-2010</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Não respiratória</t>
+          <t>Pneumonia</t>
         </is>
       </c>
       <c r="C3">
-        <v>14338</v>
+        <v>980</v>
       </c>
       <c r="D3">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2000-2010</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>SRAG</t>
         </is>
       </c>
       <c r="C4">
-        <v>2026</v>
+        <v>121</v>
       </c>
       <c r="D4">
-        <v>42.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2525,16 +2560,16 @@
         </is>
       </c>
       <c r="C5">
-        <v>2213</v>
+        <v>13497</v>
       </c>
       <c r="D5">
-        <v>46.3</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2543,16 +2578,16 @@
         </is>
       </c>
       <c r="C6">
-        <v>410</v>
+        <v>753</v>
       </c>
       <c r="D6">
-        <v>8.6</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2561,28 +2596,154 @@
         </is>
       </c>
       <c r="C7">
-        <v>133</v>
+        <v>88</v>
       </c>
       <c r="D7">
-        <v>2.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>2020-2021</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>2003</v>
+      </c>
+      <c r="D8">
+        <v>41.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2020-2021</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Não respiratória</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>2133</v>
+      </c>
+      <c r="D9">
+        <v>44.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2020-2021</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pneumonia</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>503</v>
+      </c>
+      <c r="D10">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2020-2021</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SRAG</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>143</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2022+</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>72</v>
+      </c>
+      <c r="D12">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2022+</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Não respiratória</t>
         </is>
       </c>
-      <c r="C8">
-        <v>3301</v>
-      </c>
-      <c r="D8">
-        <v>100</v>
+      <c r="C13">
+        <v>3030</v>
+      </c>
+      <c r="D13">
+        <v>91.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2022+</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pneumonia</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>161</v>
+      </c>
+      <c r="D14">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2022+</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SRAG</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>38</v>
+      </c>
+      <c r="D15">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>
@@ -2592,7 +2753,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2634,13 +2795,13 @@
         </is>
       </c>
       <c r="C2">
-        <v>2809</v>
+        <v>986</v>
       </c>
       <c r="D2">
-        <v>141936</v>
+        <v>49939</v>
       </c>
       <c r="E2">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="3">
@@ -2655,13 +2816,13 @@
         </is>
       </c>
       <c r="C3">
-        <v>2517</v>
+        <v>5769</v>
       </c>
       <c r="D3">
-        <v>127681</v>
+        <v>292055</v>
       </c>
       <c r="E3">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="4">
@@ -2672,17 +2833,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hemorragia</t>
+          <t>Doenças respiratórias (outras)</t>
         </is>
       </c>
       <c r="C4">
-        <v>4866</v>
+        <v>574</v>
       </c>
       <c r="D4">
-        <v>245711</v>
+        <v>28895</v>
       </c>
       <c r="E4">
-        <v>50.5</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="5">
@@ -2693,17 +2854,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hipertensivas</t>
+          <t>Hemorragia</t>
         </is>
       </c>
       <c r="C5">
-        <v>4520</v>
+        <v>1976</v>
       </c>
       <c r="D5">
-        <v>228743</v>
+        <v>99561</v>
       </c>
       <c r="E5">
-        <v>50.6</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="6">
@@ -2714,17 +2875,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Infecção puerperal</t>
+          <t>Hipertensivas</t>
         </is>
       </c>
       <c r="C6">
-        <v>3993</v>
+        <v>3907</v>
       </c>
       <c r="D6">
-        <v>201983</v>
+        <v>197057</v>
       </c>
       <c r="E6">
-        <v>50.6</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="7">
@@ -2735,38 +2896,38 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Outras causas diretas</t>
+          <t>Infecção puerperal</t>
         </is>
       </c>
       <c r="C7">
-        <v>874</v>
+        <v>1411</v>
       </c>
       <c r="D7">
-        <v>44573</v>
+        <v>71669</v>
       </c>
       <c r="E7">
-        <v>51</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2000-2010</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abortamento</t>
+          <t>Outras causas diretas</t>
         </is>
       </c>
       <c r="C8">
-        <v>2014</v>
+        <v>4956</v>
       </c>
       <c r="D8">
-        <v>101594</v>
+        <v>251450</v>
       </c>
       <c r="E8">
-        <v>50.4</v>
+        <v>50.7</v>
       </c>
     </row>
     <row r="9">
@@ -2777,14 +2938,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Causas indiretas</t>
+          <t>Abortamento</t>
         </is>
       </c>
       <c r="C9">
-        <v>1802</v>
+        <v>670</v>
       </c>
       <c r="D9">
-        <v>90702</v>
+        <v>33727</v>
       </c>
       <c r="E9">
         <v>50.3</v>
@@ -2798,17 +2959,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hemorragia</t>
+          <t>Causas indiretas</t>
         </is>
       </c>
       <c r="C10">
-        <v>3647</v>
+        <v>4203</v>
       </c>
       <c r="D10">
-        <v>184764</v>
+        <v>213305</v>
       </c>
       <c r="E10">
-        <v>50.7</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="11">
@@ -2819,17 +2980,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hipertensivas</t>
+          <t>Doenças respiratórias (outras)</t>
         </is>
       </c>
       <c r="C11">
-        <v>3322</v>
+        <v>450</v>
       </c>
       <c r="D11">
-        <v>168434</v>
+        <v>22695</v>
       </c>
       <c r="E11">
-        <v>50.7</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="12">
@@ -2840,17 +3001,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Infecção puerperal</t>
+          <t>Hemorragia</t>
         </is>
       </c>
       <c r="C12">
-        <v>2940</v>
+        <v>1431</v>
       </c>
       <c r="D12">
-        <v>149156</v>
+        <v>72274</v>
       </c>
       <c r="E12">
-        <v>50.7</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="13">
@@ -2861,35 +3022,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Outras causas diretas</t>
+          <t>Hipertensivas</t>
         </is>
       </c>
       <c r="C13">
-        <v>613</v>
+        <v>2864</v>
       </c>
       <c r="D13">
-        <v>31188</v>
+        <v>144630</v>
       </c>
       <c r="E13">
-        <v>50.9</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abortamento</t>
+          <t>Infecção puerperal</t>
         </is>
       </c>
       <c r="C14">
-        <v>438</v>
+        <v>1061</v>
       </c>
       <c r="D14">
-        <v>22240</v>
+        <v>53919</v>
       </c>
       <c r="E14">
         <v>50.8</v>
@@ -2898,22 +3059,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2011-2019</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>Outras causas diretas</t>
         </is>
       </c>
       <c r="C15">
-        <v>1420</v>
+        <v>3659</v>
       </c>
       <c r="D15">
-        <v>72012</v>
+        <v>185287</v>
       </c>
       <c r="E15">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="16">
@@ -2924,17 +3085,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Causas indiretas</t>
+          <t>Abortamento</t>
         </is>
       </c>
       <c r="C16">
-        <v>374</v>
+        <v>222</v>
       </c>
       <c r="D16">
-        <v>18734</v>
+        <v>11229</v>
       </c>
       <c r="E16">
-        <v>50.1</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="17">
@@ -2945,17 +3106,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Doenças respiratórias (outras)</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="C17">
-        <v>258</v>
+        <v>1421</v>
       </c>
       <c r="D17">
-        <v>12999</v>
+        <v>71960</v>
       </c>
       <c r="E17">
-        <v>50.4</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="18">
@@ -2966,17 +3127,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hemorragia</t>
+          <t>Causas indiretas</t>
         </is>
       </c>
       <c r="C18">
-        <v>849</v>
+        <v>1450</v>
       </c>
       <c r="D18">
-        <v>42898</v>
+        <v>72897</v>
       </c>
       <c r="E18">
-        <v>50.5</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="19">
@@ -2987,17 +3148,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hipertensivas</t>
+          <t>Doenças respiratórias (outras)</t>
         </is>
       </c>
       <c r="C19">
-        <v>704</v>
+        <v>257</v>
       </c>
       <c r="D19">
-        <v>35404</v>
+        <v>13051</v>
       </c>
       <c r="E19">
-        <v>50.3</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="20">
@@ -3012,13 +3173,13 @@
         </is>
       </c>
       <c r="C20">
-        <v>591</v>
+        <v>260</v>
       </c>
       <c r="D20">
-        <v>29932</v>
+        <v>13140</v>
       </c>
       <c r="E20">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="21">
@@ -3033,10 +3194,10 @@
         </is>
       </c>
       <c r="C21">
-        <v>148</v>
+        <v>1172</v>
       </c>
       <c r="D21">
-        <v>7498</v>
+        <v>59439</v>
       </c>
       <c r="E21">
         <v>50.7</v>
@@ -3054,13 +3215,13 @@
         </is>
       </c>
       <c r="C22">
-        <v>418</v>
+        <v>181</v>
       </c>
       <c r="D22">
-        <v>21413</v>
+        <v>9211</v>
       </c>
       <c r="E22">
-        <v>51.2</v>
+        <v>50.9</v>
       </c>
     </row>
     <row r="23">
@@ -3071,17 +3232,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Causas indiretas</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="C23">
-        <v>428</v>
+        <v>72</v>
       </c>
       <c r="D23">
-        <v>21765</v>
+        <v>3558</v>
       </c>
       <c r="E23">
-        <v>50.9</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="24">
@@ -3092,17 +3253,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Hemorragia</t>
+          <t>Causas indiretas</t>
         </is>
       </c>
       <c r="C24">
-        <v>823</v>
+        <v>970</v>
       </c>
       <c r="D24">
-        <v>41623</v>
+        <v>49248</v>
       </c>
       <c r="E24">
-        <v>50.6</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="25">
@@ -3113,17 +3274,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Hipertensivas</t>
+          <t>Doenças respiratórias (outras)</t>
         </is>
       </c>
       <c r="C25">
-        <v>812</v>
+        <v>100</v>
       </c>
       <c r="D25">
-        <v>41122</v>
+        <v>5031</v>
       </c>
       <c r="E25">
-        <v>50.6</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="26">
@@ -3134,17 +3295,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Infecção puerperal</t>
+          <t>Hemorragia</t>
         </is>
       </c>
       <c r="C26">
-        <v>691</v>
+        <v>304</v>
       </c>
       <c r="D26">
-        <v>34816</v>
+        <v>15397</v>
       </c>
       <c r="E26">
-        <v>50.4</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="27">
@@ -3155,17 +3316,59 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Hipertensivas</t>
+        </is>
+      </c>
+      <c r="C27">
+        <v>552</v>
+      </c>
+      <c r="D27">
+        <v>27868</v>
+      </c>
+      <c r="E27">
+        <v>50.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2022+</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Infecção puerperal</t>
+        </is>
+      </c>
+      <c r="C28">
+        <v>215</v>
+      </c>
+      <c r="D28">
+        <v>10975</v>
+      </c>
+      <c r="E28">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2022+</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Outras causas diretas</t>
         </is>
       </c>
-      <c r="C27">
-        <v>129</v>
-      </c>
-      <c r="D27">
-        <v>6659</v>
-      </c>
-      <c r="E27">
-        <v>51.6</v>
+      <c r="C29">
+        <v>907</v>
+      </c>
+      <c r="D29">
+        <v>46109</v>
+      </c>
+      <c r="E29">
+        <v>50.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>